<commit_message>
paper review: drop reliability and note columns from Canva export
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TW26B3fiA9YvDmaURBJTqZ
</commit_message>
<xml_diff>
--- a/poc/Finding Dataset/paper review/export/summary.xlsx
+++ b/poc/Finding Dataset/paper review/export/summary.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,18 +29,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="000D6B69"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="008A5300"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00B3261E"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,21 +56,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -451,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -463,8 +442,6 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,16 +490,6 @@
           <t>วัดผลการแชร์ได้ไหม</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>ความน่าเชื่อถือ</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>หมายเหตุ</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -570,16 +537,6 @@
           <t>ได้: +22 จุด</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>ดี</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>มีแค่ accuracy</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -627,16 +584,6 @@
           <t>ได้: +0.026</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>กลาง</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>ข้อความขัดกับกราฟ</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -684,12 +631,6 @@
           <t>ได้: DR → 90.5–98.6%</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>ดี</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -737,16 +678,6 @@
           <t>ได้: FedAvg ≈0.36 แย่กว่าเดี่ยว</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>ดี</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>อ่านจาก box plot</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -794,12 +725,6 @@
           <t>ไม่ได้ (เทียบ DFL ≥ CFL ได้)</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>ดี</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -847,16 +772,6 @@
           <t>ไม่ได้</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>กลาง</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>preprint</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -904,12 +819,6 @@
           <t>ไม่ได้</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>กลาง</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -957,16 +866,6 @@
           <t>ไม่ได้</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>ต่ำ</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>ตาราง 0.97 vs เนื้อหา 85.31%</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1014,16 +913,6 @@
           <t>ไม่ได้</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>ต่ำ</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>recall ของคลาส 0.006% ได้ 98%</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1071,16 +960,6 @@
           <t>ไม่ได้</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>ต่ำ</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>ไม่ระบุโมเดล</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1128,12 +1007,6 @@
           <t>ไม่ได้</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>ต่ำ</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1179,16 +1052,6 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>–</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>ไม่ทราบ</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>ไฟล์ที่อัปโหลดเป็น paper MRI</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1074,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ประเด็น</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>จำนวน</t>
         </is>

</xml_diff>